<commit_message>
Added ensemble docking evaluation and metrics - CLI version
</commit_message>
<xml_diff>
--- a/templates/anathi_template.xlsx
+++ b/templates/anathi_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anathimsobo/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gerritkoorsen/docking_platform_gui/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D08F25D2-FA01-4A40-9216-F7B9C3E65734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2261DDDA-2D41-A04C-9D1D-F1E22D6EA113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="69">
   <si>
     <t>Protein</t>
   </si>
@@ -221,13 +221,19 @@
   </si>
   <si>
     <t>MYC</t>
+  </si>
+  <si>
+    <t>SMILES</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -242,6 +248,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF111827"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -279,11 +291,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,16 +601,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.5" customWidth="1"/>
-    <col min="5" max="5" width="29.1640625" customWidth="1"/>
-    <col min="6" max="6" width="23.83203125" customWidth="1"/>
-    <col min="7" max="7" width="70" customWidth="1"/>
+    <col min="6" max="6" width="29.1640625" customWidth="1"/>
+    <col min="7" max="7" width="23.83203125" customWidth="1"/>
+    <col min="8" max="8" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -611,16 +624,19 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -630,34 +646,40 @@
       <c r="D2" t="s">
         <v>27</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" t="s">
         <v>28</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>34</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" t="s">
         <v>28</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -671,16 +693,19 @@
         <v>62</v>
       </c>
       <c r="E4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>36</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -694,101 +719,119 @@
         <v>63</v>
       </c>
       <c r="E5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" t="s">
         <v>30</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>37</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F6" t="s">
         <v>28</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>38</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F7" t="s">
         <v>28</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>39</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" t="s">
         <v>28</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>40</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F9" t="s">
         <v>28</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>41</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>7</v>
       </c>
       <c r="B10" t="s">
         <v>16</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" t="s">
         <v>28</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>42</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -801,34 +844,40 @@
       <c r="D11" t="s">
         <v>64</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" t="s">
         <v>31</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>43</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>7</v>
       </c>
       <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" t="s">
         <v>28</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -841,34 +890,40 @@
       <c r="D13" t="s">
         <v>65</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" t="s">
         <v>32</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>45</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>7</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" t="s">
         <v>28</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>46</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -881,13 +936,16 @@
       <c r="D15" t="s">
         <v>66</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" t="s">
         <v>33</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>47</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>61</v>
       </c>
     </row>

</xml_diff>